<commit_message>
fix: sanitize OKVED XLSX downloads
</commit_message>
<xml_diff>
--- a/data/processed/okved/downloads/okved-20-41-moscow-oblast.xlsx
+++ b/data/processed/okved/downloads/okved-20-41-moscow-oblast.xlsx
@@ -12793,10 +12793,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="OKVED 20.41 Moscow + Oblst" connectionId="1" xr16:uid="{0D5CB7C3-C9BC-3C46-A441-421A9640CD99}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>